<commit_message>
Summary leads with Generative AI feature impressions
</commit_message>
<xml_diff>
--- a/examples/sample-report.xlsx
+++ b/examples/sample-report.xlsx
@@ -11340,7 +11340,7 @@
       </c>
       <c r="F6" s="19" t="inlineStr">
         <is>
-          <t>Flake questions rank 2.9-9.1 and the flake page is the second most AI-shown page (1,189 AI impressions). 'What is flake epoxy flooring' ranks 2.9 with low CTR: the AI answer is summarising it.</t>
+          <t>Flake questions rank 2.5-9.1 and the flake page is the second most AI-shown page (1,189 AI impressions). 'What is flake epoxy flooring' ranks 2.9 with low CTR: the AI answer is summarising it.</t>
         </is>
       </c>
       <c r="G6" s="19" t="inlineStr">
@@ -11833,7 +11833,7 @@
       </c>
       <c r="F13" s="19" t="inlineStr">
         <is>
-          <t>Five AI Mode follow-ups with no topic word: 'show me photos', 'which is cheaper?', 'how about in brisbane', 'are they slippery'. People are mid-conversation with Google's AI and want pictures, prices and a nearby option.</t>
+          <t>Four AI Mode follow-ups with no topic word: 'show me photos', 'which is cheaper?', 'how about in brisbane', 'are they slippery'. People are mid-conversation with Google's AI and want pictures, prices and a nearby option.</t>
         </is>
       </c>
       <c r="G13" s="19" t="inlineStr"/>

</xml_diff>